<commit_message>
Vanilla Plants Expanded - Flowers 업데이트
Co-Authored-By: DeaD DooDle <33118840+basalt991@users.noreply.github.com>

#3043
</commit_message>
<xml_diff>
--- a/Data/Vanilla Expanded/Vanilla Plants Expanded - Flowers - 3748351639/1.6/Vanilla Plants Expanded - Flowers - 3748351639.xlsx
+++ b/Data/Vanilla Expanded/Vanilla Plants Expanded - Flowers - 3748351639/1.6/Vanilla Plants Expanded - Flowers - 3748351639.xlsx
@@ -8,7 +8,8 @@
     <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
   </bookViews>
   <sheets>
-    <sheet name="Current_260621" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="Current_260710" sheetId="1" state="visible" r:id="rId3"/>
+    <sheet name="260621" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -20,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="250">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="672" uniqueCount="299">
   <si>
     <t xml:space="preserve">Class+Node [(Identifier (Key)]</t>
   </si>
@@ -754,22 +755,169 @@
     <t xml:space="preserve">VPE_BloomingFlowerZone</t>
   </si>
   <si>
+    <t xml:space="preserve">Blooming flower zone</t>
+  </si>
+  <si>
+    <t xml:space="preserve">꽃밭 구역</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Keyed+VPE_BloomingFlowerZoneDesc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VPE_BloomingFlowerZoneDesc</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Create a zone where your colonists will try to grow blooming flowers.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">정착민들이 꽃을 재배할 구역을 만듭니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ThingDef+VPEF_Plant_BeardedIris.label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VPEF_Plant_BeardedIris.label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bearded iris</t>
+  </si>
+  <si>
+    <t xml:space="preserve">수염붓꽃</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ThingDef+VPEF_Plant_BeardedIris.description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VPEF_Plant_BeardedIris.description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A distinct perennial known for its unique, beard-like hairs on the lower petals of its large, elegant flowers. It creates a stunning visual display and grows in large clusters.\n\nBlooms from 1st day of spring to 5th day of summer.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">크고 우아한 꽃의 아래쪽 꽃잎에 수염처럼 난 독특한 털로 잘 알려진 다년생 식물입니다. 무리 지어 자라며 화려한 경관을 이룹니다.\n\n봄 1일부터 여름 5일까지 꽃을 피웁니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ThingDef+VPEF_Plant_FlameAzalea.label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VPEF_Plant_FlameAzalea.label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">flame azalea bush</t>
+  </si>
+  <si>
+    <t xml:space="preserve">불꽃철쭉 덤불</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ThingDef+VPEF_Plant_FlameAzalea.description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VPEF_Plant_FlameAzalea.description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A striking, deciduous shrub known for its brilliant, flame-orange clusters of tubular flowers. It thrives in acidic soils and provides a vibrant, fire-like visual contrast in any garden.\n\nBlooms from 5th day of spring to 10th day of summer.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">불꽃 같은 주황색의 관 모양 꽃이 무리 지어 피는 인상적인 낙엽성 관목입니다. 산성 토양에서 잘 자라며, 어떤 정원에서든 불꽃 같은 선명한 대비를 더합니다.\n\n봄 5일부터 여름 10일까지 꽃을 피웁니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ThingDef+VPEF_Plant_PampasGrass.label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VPEF_Plant_PampasGrass.label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pampas grass</t>
+  </si>
+  <si>
+    <t xml:space="preserve">팜파스그래스</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ThingDef+VPEF_Plant_PampasGrass.description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VPEF_Plant_PampasGrass.description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A tall, vigorous ornamental grass famous for its large, feathery white plumes that sway in the wind. It provides structure and height to garden borders and is remarkably resilient.\n\nBlooms from 1st day of summer to 15th day of fall.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">바람에 흔들리는 크고 깃털 같은 흰 꽃차례로 유명한 키 큰 장식용 풀입니다. 정원 가장자리에 구조감과 높이감을 더해주며 매우 강인합니다.\n\n여름 1일부터 가을 15일까지 꽃을 피웁니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ThingDef+VPEF_Plant_PraireFire.label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VPEF_Plant_PraireFire.label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">prairie fire</t>
+  </si>
+  <si>
+    <t xml:space="preserve">프레리 파이어</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ThingDef+VPEF_Plant_PraireFire.description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VPEF_Plant_PraireFire.description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A hardy, vibrant flower known for its fiery red and orange petals that resemble dancing flames. It is exceptionally resilient and thrives in hot, sunny conditions.\n\nBlooms from 5th day of summer to 10th day of fall.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">춤추는 불꽃을 닮은 강렬한 붉은색과 주황색 꽃잎으로 잘 알려진 강인하고 화려한 꽃입니다. 척박한 환경에도 잘 견디며, 덥고 햇볕이 잘 드는 환경에서 잘 자랍니다.\n\n여름 5일부터 가을 10일까지 꽃을 피웁니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ThingDef+VPEF_Plant_Bloomaris.label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VPEF_Plant_Bloomaris.label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bloomaris</t>
+  </si>
+  <si>
+    <t xml:space="preserve">블루마리스</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ThingDef+VPEF_Plant_Bloomaris.description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VPEF_Plant_Bloomaris.description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">An exotic, decorative fungus that can be grown in caves. It thrives in almost total darkness, emitting a soft, warm glow.\n\nBlooms almost continuously, but only when the light level is below 20%. It will die if temperature falls below -26C.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">동굴에서 재배할 수 있는 이국적인 장식용 균류입니다. 거의 빛이 없는 어둠 속에서 잘 자라며 은은하고 따뜻한 빛을 냅니다.\n\n거의 계속 꽃을 피우지만, 밝기가 20% 미만일 때만 가능합니다. 온도가 -26C 아래로 내려가면 죽습니다.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ThingDef+VPEF_Plant_PinkCyclamen.label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VPEF_Plant_PinkCyclamen.label</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pink cyclamen</t>
+  </si>
+  <si>
+    <t xml:space="preserve">분홍 시클라멘</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ThingDef+VPEF_Plant_PinkCyclamen.description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VPEF_Plant_PinkCyclamen.description</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A delicate, low-growing perennial with swept-back petals that seem to dance in the breeze. They prefer cooler temperatures and will not bloom if it’s too hot.\n\nBlooms from 10th day of fall to 10th day of spring.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">바람에 춤추는 듯 뒤로 젖혀진 꽃잎을 가진 섬세하고 키 작은 다년생 식물입니다. 서늘한 온도를 선호하며 너무 더우면 꽃을 피우지 않습니다.\n\n가을 10일부터 봄 10일까지 꽃을 피웁니다.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Blooming Flower Zone</t>
-  </si>
-  <si>
-    <t xml:space="preserve">꽃밭 구역</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Keyed+VPE_BloomingFlowerZoneDesc</t>
-  </si>
-  <si>
-    <t xml:space="preserve">VPE_BloomingFlowerZoneDesc</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Create a zone where your colonists will try to grow blooming flowers.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">정착민들이 꽃을 재배할 구역을 만듭니다.</t>
   </si>
 </sst>
 </file>
@@ -852,8 +1000,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="4">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -881,34 +1037,34 @@
         <a:srgbClr val="000000"/>
       </a:dk1>
       <a:lt1>
-        <a:srgbClr val="ffffff"/>
+        <a:srgbClr val="FFFFFF"/>
       </a:lt1>
       <a:dk2>
-        <a:srgbClr val="1f497d"/>
+        <a:srgbClr val="1F497D"/>
       </a:dk2>
       <a:lt2>
-        <a:srgbClr val="eeece1"/>
+        <a:srgbClr val="EEECE1"/>
       </a:lt2>
       <a:accent1>
-        <a:srgbClr val="4f81bd"/>
+        <a:srgbClr val="4F81BD"/>
       </a:accent1>
       <a:accent2>
-        <a:srgbClr val="c0504d"/>
+        <a:srgbClr val="C0504D"/>
       </a:accent2>
       <a:accent3>
-        <a:srgbClr val="9bbb59"/>
+        <a:srgbClr val="9BBB59"/>
       </a:accent3>
       <a:accent4>
-        <a:srgbClr val="8064a2"/>
+        <a:srgbClr val="8064A2"/>
       </a:accent4>
       <a:accent5>
-        <a:srgbClr val="4bacc6"/>
+        <a:srgbClr val="4BACC6"/>
       </a:accent5>
       <a:accent6>
-        <a:srgbClr val="f79646"/>
+        <a:srgbClr val="F79646"/>
       </a:accent6>
       <a:hlink>
-        <a:srgbClr val="0000ff"/>
+        <a:srgbClr val="0000FF"/>
       </a:hlink>
       <a:folHlink>
         <a:srgbClr val="800080"/>
@@ -1053,1054 +1209,2325 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F61"/>
-  <sheetFormatPr defaultColWidth="8.390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:F73"/>
+  <sheetFormatPr defaultColWidth="8.390625" defaultRowHeight="13.8" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44.09"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="17.25"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="34.07"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="25.46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="87.64"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="44.09"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="17.25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="34.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="25.46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="63.53"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="7" style="1" width="8.39"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="0" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="0" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="0" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="0" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="0" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="0" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
     </row>
+    <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="3" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F10" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="E12" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="1" t="s">
+        <v>57</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="E13" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="E14" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E15" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="E16" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="E17" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="E18" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="1" t="s">
+        <v>81</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="E20" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="E21" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="E22" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="E23" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>102</v>
+      </c>
+      <c r="E24" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="E25" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="E26" s="1" t="s">
+        <v>111</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="E27" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="E28" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="1" t="s">
+        <v>121</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="E29" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>126</v>
+      </c>
+      <c r="E30" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="E31" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="1" t="s">
+        <v>133</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="E32" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="E33" s="1" t="s">
+        <v>139</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="1" t="s">
+        <v>141</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="E34" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>146</v>
+      </c>
+      <c r="E35" s="1" t="s">
+        <v>147</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="1" t="s">
+        <v>149</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="E36" s="1" t="s">
+        <v>151</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="E37" s="1" t="s">
+        <v>155</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="1" t="s">
+        <v>157</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>158</v>
+      </c>
+      <c r="E38" s="1" t="s">
+        <v>159</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>162</v>
+      </c>
+      <c r="E39" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="F39" s="1" t="s">
+        <v>164</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="1" t="s">
+        <v>165</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>166</v>
+      </c>
+      <c r="E40" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="F40" s="1" t="s">
+        <v>168</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="1" t="s">
+        <v>169</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="E41" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="F41" s="1" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="1" t="s">
+        <v>173</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>174</v>
+      </c>
+      <c r="E42" s="1" t="s">
+        <v>175</v>
+      </c>
+      <c r="F42" s="1" t="s">
+        <v>176</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="E43" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="F43" s="1" t="s">
+        <v>180</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="E44" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="F44" s="1" t="s">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="1" t="s">
+        <v>185</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>186</v>
+      </c>
+      <c r="E45" s="1" t="s">
+        <v>187</v>
+      </c>
+      <c r="F45" s="1" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="1" t="s">
+        <v>189</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>190</v>
+      </c>
+      <c r="E46" s="1" t="s">
+        <v>191</v>
+      </c>
+      <c r="F46" s="1" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="1" t="s">
+        <v>193</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>194</v>
+      </c>
+      <c r="E47" s="1" t="s">
+        <v>195</v>
+      </c>
+      <c r="F47" s="1" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>198</v>
+      </c>
+      <c r="E48" s="1" t="s">
+        <v>199</v>
+      </c>
+      <c r="F48" s="1" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="1" t="s">
+        <v>201</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C49" s="1" t="s">
+        <v>202</v>
+      </c>
+      <c r="E49" s="1" t="s">
+        <v>203</v>
+      </c>
+      <c r="F49" s="1" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="1" t="s">
+        <v>205</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>206</v>
+      </c>
+      <c r="E50" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="F50" s="1" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="1" t="s">
+        <v>209</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C51" s="1" t="s">
+        <v>210</v>
+      </c>
+      <c r="E51" s="1" t="s">
+        <v>211</v>
+      </c>
+      <c r="F51" s="1" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="1" t="s">
+        <v>213</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="C52" s="1" t="s">
+        <v>215</v>
+      </c>
+      <c r="E52" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="F52" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="1" t="s">
+        <v>216</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>214</v>
+      </c>
+      <c r="C53" s="1" t="s">
+        <v>217</v>
+      </c>
+      <c r="E53" s="1" t="s">
+        <v>218</v>
+      </c>
+      <c r="F53" s="1" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="1" t="s">
+        <v>220</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>222</v>
+      </c>
+      <c r="E54" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="F54" s="1" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>226</v>
+      </c>
+      <c r="E55" s="1" t="s">
+        <v>223</v>
+      </c>
+      <c r="F55" s="1" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="1" t="s">
+        <v>227</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>228</v>
+      </c>
+      <c r="E56" s="1" t="s">
+        <v>229</v>
+      </c>
+      <c r="F56" s="1" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="E57" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="F57" s="1" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="1" t="s">
+        <v>235</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="C58" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="E58" s="1" t="s">
+        <v>233</v>
+      </c>
+      <c r="F58" s="1" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>221</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="E59" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="F59" s="1" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="1" t="s">
+        <v>241</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>243</v>
+      </c>
+      <c r="E60" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="F60" s="1" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="61" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="1" t="s">
+        <v>246</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="C61" s="1" t="s">
+        <v>247</v>
+      </c>
+      <c r="E61" s="1" t="s">
+        <v>248</v>
+      </c>
+      <c r="F61" s="1" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="1" t="s">
+        <v>250</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>251</v>
+      </c>
+      <c r="E62" s="1" t="s">
+        <v>252</v>
+      </c>
+      <c r="F62" s="1" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C63" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="E63" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="F63" s="1" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C64" s="1" t="s">
+        <v>259</v>
+      </c>
+      <c r="E64" s="1" t="s">
+        <v>260</v>
+      </c>
+      <c r="F64" s="1" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C65" s="1" t="s">
+        <v>263</v>
+      </c>
+      <c r="E65" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="F65" s="1" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="E66" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="F66" s="1" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A67" s="1" t="s">
+        <v>270</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C67" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="E67" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="F67" s="1" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C68" s="1" t="s">
+        <v>275</v>
+      </c>
+      <c r="E68" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="F68" s="1" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C69" s="1" t="s">
+        <v>279</v>
+      </c>
+      <c r="E69" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="F69" s="1" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C70" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="E70" s="1" t="s">
+        <v>284</v>
+      </c>
+      <c r="F70" s="1" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C71" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="E71" s="1" t="s">
+        <v>288</v>
+      </c>
+      <c r="F71" s="1" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="1" t="s">
+        <v>290</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C72" s="1" t="s">
+        <v>291</v>
+      </c>
+      <c r="E72" s="1" t="s">
+        <v>292</v>
+      </c>
+      <c r="F72" s="1" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A73" s="1" t="s">
+        <v>294</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C73" s="1" t="s">
+        <v>295</v>
+      </c>
+      <c r="E73" s="1" t="s">
+        <v>296</v>
+      </c>
+      <c r="F73" s="1" t="s">
+        <v>297</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader>&amp;C&amp;"Times New Roman,보통"&amp;12&amp;Kffffff&amp;A</oddHeader>
+    <oddFooter>&amp;C&amp;"Times New Roman,보통"&amp;12&amp;Kffffff페이지 &amp;P</oddFooter>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:F61"/>
+  <sheetFormatPr defaultColWidth="8.390625" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="44.09"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="2" width="17.25"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="2" width="34.07"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="2" width="25.46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="2" width="87.64"/>
+    <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="7" style="3" width="8.39"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>5</v>
+      </c>
+    </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="s">
+      <c r="A2" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="0" t="s">
+      <c r="E2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="0" t="s">
+      <c r="F2" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="s">
+      <c r="A3" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E3" s="0" t="s">
+      <c r="E3" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F3" s="0" t="s">
+      <c r="F3" s="2" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="s">
+      <c r="A4" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="0" t="s">
+      <c r="B4" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C4" s="0" t="s">
+      <c r="C4" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="E4" s="0" t="s">
+      <c r="E4" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="F4" s="0" t="s">
+      <c r="F4" s="2" t="s">
         <v>19</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="s">
+      <c r="A5" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B5" s="0" t="s">
+      <c r="B5" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C5" s="0" t="s">
+      <c r="C5" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="E5" s="0" t="s">
+      <c r="E5" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="F5" s="0" t="s">
+      <c r="F5" s="2" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="s">
+      <c r="A6" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B6" s="0" t="s">
+      <c r="B6" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C6" s="0" t="s">
+      <c r="C6" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="E6" s="0" t="s">
+      <c r="E6" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="F6" s="0" t="s">
+      <c r="F6" s="2" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="s">
+      <c r="A7" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="B7" s="0" t="s">
+      <c r="B7" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C7" s="0" t="s">
+      <c r="C7" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="E7" s="0" t="s">
+      <c r="E7" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="F7" s="0" t="s">
+      <c r="F7" s="2" t="s">
         <v>34</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="s">
+      <c r="A8" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="B8" s="0" t="s">
+      <c r="B8" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C8" s="0" t="s">
+      <c r="C8" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="E8" s="0" t="s">
+      <c r="E8" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="F8" s="0" t="s">
+      <c r="F8" s="2" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="s">
+      <c r="A9" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="C9" s="0" t="s">
+      <c r="C9" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="E9" s="0" t="s">
+      <c r="E9" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="F9" s="0" t="s">
+      <c r="F9" s="2" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="s">
+      <c r="A10" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="B10" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="C10" s="0" t="s">
+      <c r="B10" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C10" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="E10" s="0" t="s">
+      <c r="E10" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="F10" s="0" t="s">
+      <c r="F10" s="2" t="s">
         <v>48</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="0" t="s">
+      <c r="A11" s="2" t="s">
         <v>49</v>
       </c>
-      <c r="B11" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="C11" s="0" t="s">
+      <c r="B11" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C11" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="E11" s="0" t="s">
+      <c r="E11" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="F11" s="0" t="s">
+      <c r="F11" s="2" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="0" t="s">
+      <c r="A12" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B12" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="C12" s="0" t="s">
+      <c r="B12" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C12" s="2" t="s">
         <v>54</v>
       </c>
-      <c r="E12" s="0" t="s">
+      <c r="E12" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="F12" s="0" t="s">
+      <c r="F12" s="2" t="s">
         <v>56</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="0" t="s">
+      <c r="A13" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B13" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="C13" s="0" t="s">
+      <c r="B13" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C13" s="2" t="s">
         <v>58</v>
       </c>
-      <c r="E13" s="0" t="s">
+      <c r="E13" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="F13" s="0" t="s">
+      <c r="F13" s="2" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="0" t="s">
+      <c r="A14" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B14" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="C14" s="0" t="s">
+      <c r="B14" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C14" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="E14" s="0" t="s">
+      <c r="E14" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="F14" s="0" t="s">
+      <c r="F14" s="2" t="s">
         <v>64</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="0" t="s">
+      <c r="A15" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="B15" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="C15" s="0" t="s">
+      <c r="B15" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C15" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="E15" s="0" t="s">
+      <c r="E15" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="F15" s="0" t="s">
+      <c r="F15" s="2" t="s">
         <v>68</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="0" t="s">
+      <c r="A16" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="B16" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="C16" s="0" t="s">
+      <c r="B16" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="E16" s="0" t="s">
+      <c r="E16" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="F16" s="0" t="s">
+      <c r="F16" s="2" t="s">
         <v>72</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="0" t="s">
+      <c r="A17" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="B17" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="C17" s="0" t="s">
+      <c r="B17" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>74</v>
       </c>
-      <c r="E17" s="0" t="s">
+      <c r="E17" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="F17" s="0" t="s">
+      <c r="F17" s="2" t="s">
         <v>76</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="0" t="s">
+      <c r="A18" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="B18" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="C18" s="0" t="s">
+      <c r="B18" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C18" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="E18" s="0" t="s">
+      <c r="E18" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="F18" s="0" t="s">
+      <c r="F18" s="2" t="s">
         <v>80</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="0" t="s">
+      <c r="A19" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="B19" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="C19" s="0" t="s">
+      <c r="B19" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>82</v>
       </c>
-      <c r="E19" s="0" t="s">
+      <c r="E19" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="F19" s="0" t="s">
+      <c r="F19" s="2" t="s">
         <v>84</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="0" t="s">
+      <c r="A20" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="B20" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="C20" s="0" t="s">
+      <c r="B20" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C20" s="2" t="s">
         <v>86</v>
       </c>
-      <c r="E20" s="0" t="s">
+      <c r="E20" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="F20" s="0" t="s">
+      <c r="F20" s="2" t="s">
         <v>88</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="0" t="s">
+      <c r="A21" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="B21" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="C21" s="0" t="s">
+      <c r="B21" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C21" s="2" t="s">
         <v>90</v>
       </c>
-      <c r="E21" s="0" t="s">
+      <c r="E21" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="F21" s="0" t="s">
+      <c r="F21" s="2" t="s">
         <v>92</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="0" t="s">
+      <c r="A22" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B22" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="C22" s="0" t="s">
+      <c r="B22" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C22" s="2" t="s">
         <v>94</v>
       </c>
-      <c r="E22" s="0" t="s">
+      <c r="E22" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="F22" s="0" t="s">
+      <c r="F22" s="2" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="0" t="s">
+      <c r="A23" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="B23" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="C23" s="0" t="s">
+      <c r="B23" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C23" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="E23" s="0" t="s">
+      <c r="E23" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="F23" s="0" t="s">
+      <c r="F23" s="2" t="s">
         <v>100</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="0" t="s">
+      <c r="A24" s="2" t="s">
         <v>101</v>
       </c>
-      <c r="B24" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="C24" s="0" t="s">
+      <c r="B24" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C24" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="E24" s="0" t="s">
+      <c r="E24" s="2" t="s">
         <v>103</v>
       </c>
-      <c r="F24" s="0" t="s">
+      <c r="F24" s="2" t="s">
         <v>104</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="0" t="s">
+      <c r="A25" s="2" t="s">
         <v>105</v>
       </c>
-      <c r="B25" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="C25" s="0" t="s">
+      <c r="B25" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C25" s="2" t="s">
         <v>106</v>
       </c>
-      <c r="E25" s="0" t="s">
+      <c r="E25" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="F25" s="0" t="s">
+      <c r="F25" s="2" t="s">
         <v>108</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="0" t="s">
+      <c r="A26" s="2" t="s">
         <v>109</v>
       </c>
-      <c r="B26" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="C26" s="0" t="s">
+      <c r="B26" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C26" s="2" t="s">
         <v>110</v>
       </c>
-      <c r="E26" s="0" t="s">
+      <c r="E26" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="F26" s="0" t="s">
+      <c r="F26" s="2" t="s">
         <v>112</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="0" t="s">
+      <c r="A27" s="2" t="s">
         <v>113</v>
       </c>
-      <c r="B27" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="C27" s="0" t="s">
+      <c r="B27" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C27" s="2" t="s">
         <v>114</v>
       </c>
-      <c r="E27" s="0" t="s">
+      <c r="E27" s="2" t="s">
         <v>115</v>
       </c>
-      <c r="F27" s="0" t="s">
+      <c r="F27" s="2" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="0" t="s">
+      <c r="A28" s="2" t="s">
         <v>117</v>
       </c>
-      <c r="B28" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="C28" s="0" t="s">
+      <c r="B28" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C28" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="E28" s="0" t="s">
+      <c r="E28" s="2" t="s">
         <v>119</v>
       </c>
-      <c r="F28" s="0" t="s">
+      <c r="F28" s="2" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="0" t="s">
+      <c r="A29" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="B29" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="C29" s="0" t="s">
+      <c r="B29" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C29" s="2" t="s">
         <v>122</v>
       </c>
-      <c r="E29" s="0" t="s">
+      <c r="E29" s="2" t="s">
         <v>123</v>
       </c>
-      <c r="F29" s="0" t="s">
+      <c r="F29" s="2" t="s">
         <v>124</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="0" t="s">
+      <c r="A30" s="2" t="s">
         <v>125</v>
       </c>
-      <c r="B30" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="C30" s="0" t="s">
+      <c r="B30" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C30" s="2" t="s">
         <v>126</v>
       </c>
-      <c r="E30" s="0" t="s">
+      <c r="E30" s="2" t="s">
         <v>127</v>
       </c>
-      <c r="F30" s="0" t="s">
+      <c r="F30" s="2" t="s">
         <v>128</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="0" t="s">
+      <c r="A31" s="2" t="s">
         <v>129</v>
       </c>
-      <c r="B31" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="C31" s="0" t="s">
+      <c r="B31" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C31" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="E31" s="0" t="s">
+      <c r="E31" s="2" t="s">
         <v>131</v>
       </c>
-      <c r="F31" s="0" t="s">
+      <c r="F31" s="2" t="s">
         <v>132</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="0" t="s">
+      <c r="A32" s="2" t="s">
         <v>133</v>
       </c>
-      <c r="B32" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="C32" s="0" t="s">
+      <c r="B32" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C32" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="E32" s="0" t="s">
+      <c r="E32" s="2" t="s">
         <v>135</v>
       </c>
-      <c r="F32" s="0" t="s">
+      <c r="F32" s="2" t="s">
         <v>136</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="0" t="s">
+      <c r="A33" s="2" t="s">
         <v>137</v>
       </c>
-      <c r="B33" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="C33" s="0" t="s">
+      <c r="B33" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C33" s="2" t="s">
         <v>138</v>
       </c>
-      <c r="E33" s="0" t="s">
+      <c r="E33" s="2" t="s">
         <v>139</v>
       </c>
-      <c r="F33" s="0" t="s">
+      <c r="F33" s="2" t="s">
         <v>140</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="0" t="s">
+      <c r="A34" s="2" t="s">
         <v>141</v>
       </c>
-      <c r="B34" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="C34" s="0" t="s">
+      <c r="B34" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C34" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="E34" s="0" t="s">
+      <c r="E34" s="2" t="s">
         <v>143</v>
       </c>
-      <c r="F34" s="0" t="s">
+      <c r="F34" s="2" t="s">
         <v>144</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="0" t="s">
+      <c r="A35" s="2" t="s">
         <v>145</v>
       </c>
-      <c r="B35" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="C35" s="0" t="s">
+      <c r="B35" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C35" s="2" t="s">
         <v>146</v>
       </c>
-      <c r="E35" s="0" t="s">
+      <c r="E35" s="2" t="s">
         <v>147</v>
       </c>
-      <c r="F35" s="0" t="s">
+      <c r="F35" s="2" t="s">
         <v>148</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="0" t="s">
+      <c r="A36" s="2" t="s">
         <v>149</v>
       </c>
-      <c r="B36" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="C36" s="0" t="s">
+      <c r="B36" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C36" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="E36" s="0" t="s">
+      <c r="E36" s="2" t="s">
         <v>151</v>
       </c>
-      <c r="F36" s="0" t="s">
+      <c r="F36" s="2" t="s">
         <v>152</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="0" t="s">
+      <c r="A37" s="2" t="s">
         <v>153</v>
       </c>
-      <c r="B37" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="C37" s="0" t="s">
+      <c r="B37" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C37" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="E37" s="0" t="s">
+      <c r="E37" s="2" t="s">
         <v>155</v>
       </c>
-      <c r="F37" s="0" t="s">
+      <c r="F37" s="2" t="s">
         <v>156</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="0" t="s">
+      <c r="A38" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="B38" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="C38" s="0" t="s">
+      <c r="B38" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C38" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="E38" s="0" t="s">
+      <c r="E38" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="F38" s="0" t="s">
+      <c r="F38" s="2" t="s">
         <v>160</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="0" t="s">
+      <c r="A39" s="2" t="s">
         <v>161</v>
       </c>
-      <c r="B39" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="C39" s="0" t="s">
+      <c r="B39" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C39" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="E39" s="0" t="s">
+      <c r="E39" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="F39" s="0" t="s">
+      <c r="F39" s="2" t="s">
         <v>164</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="0" t="s">
+      <c r="A40" s="2" t="s">
         <v>165</v>
       </c>
-      <c r="B40" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="C40" s="0" t="s">
+      <c r="B40" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C40" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="E40" s="0" t="s">
+      <c r="E40" s="2" t="s">
         <v>167</v>
       </c>
-      <c r="F40" s="0" t="s">
+      <c r="F40" s="2" t="s">
         <v>168</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="0" t="s">
+      <c r="A41" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="B41" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="C41" s="0" t="s">
+      <c r="B41" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C41" s="2" t="s">
         <v>170</v>
       </c>
-      <c r="E41" s="0" t="s">
+      <c r="E41" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="F41" s="0" t="s">
+      <c r="F41" s="2" t="s">
         <v>172</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="0" t="s">
+      <c r="A42" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="B42" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="C42" s="0" t="s">
+      <c r="B42" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C42" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="E42" s="0" t="s">
+      <c r="E42" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="F42" s="0" t="s">
+      <c r="F42" s="2" t="s">
         <v>176</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="0" t="s">
+      <c r="A43" s="2" t="s">
         <v>177</v>
       </c>
-      <c r="B43" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="C43" s="0" t="s">
+      <c r="B43" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C43" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="E43" s="0" t="s">
+      <c r="E43" s="2" t="s">
         <v>179</v>
       </c>
-      <c r="F43" s="0" t="s">
+      <c r="F43" s="2" t="s">
         <v>180</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="0" t="s">
+      <c r="A44" s="2" t="s">
         <v>181</v>
       </c>
-      <c r="B44" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="C44" s="0" t="s">
+      <c r="B44" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C44" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="E44" s="0" t="s">
+      <c r="E44" s="2" t="s">
         <v>183</v>
       </c>
-      <c r="F44" s="0" t="s">
+      <c r="F44" s="2" t="s">
         <v>184</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="0" t="s">
+      <c r="A45" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="B45" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="C45" s="0" t="s">
+      <c r="B45" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C45" s="2" t="s">
         <v>186</v>
       </c>
-      <c r="E45" s="0" t="s">
+      <c r="E45" s="2" t="s">
         <v>187</v>
       </c>
-      <c r="F45" s="0" t="s">
+      <c r="F45" s="2" t="s">
         <v>188</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="0" t="s">
+      <c r="A46" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="B46" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="C46" s="0" t="s">
+      <c r="B46" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C46" s="2" t="s">
         <v>190</v>
       </c>
-      <c r="E46" s="0" t="s">
+      <c r="E46" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="F46" s="0" t="s">
+      <c r="F46" s="2" t="s">
         <v>192</v>
       </c>
     </row>
     <row r="47" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="0" t="s">
+      <c r="A47" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="B47" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="C47" s="0" t="s">
+      <c r="B47" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C47" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="E47" s="0" t="s">
+      <c r="E47" s="2" t="s">
         <v>195</v>
       </c>
-      <c r="F47" s="0" t="s">
+      <c r="F47" s="2" t="s">
         <v>196</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="0" t="s">
+      <c r="A48" s="2" t="s">
         <v>197</v>
       </c>
-      <c r="B48" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="C48" s="0" t="s">
+      <c r="B48" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C48" s="2" t="s">
         <v>198</v>
       </c>
-      <c r="E48" s="0" t="s">
+      <c r="E48" s="2" t="s">
         <v>199</v>
       </c>
-      <c r="F48" s="0" t="s">
+      <c r="F48" s="2" t="s">
         <v>200</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="0" t="s">
+      <c r="A49" s="2" t="s">
         <v>201</v>
       </c>
-      <c r="B49" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="C49" s="0" t="s">
+      <c r="B49" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C49" s="2" t="s">
         <v>202</v>
       </c>
-      <c r="E49" s="0" t="s">
+      <c r="E49" s="2" t="s">
         <v>203</v>
       </c>
-      <c r="F49" s="0" t="s">
+      <c r="F49" s="2" t="s">
         <v>204</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="0" t="s">
+      <c r="A50" s="2" t="s">
         <v>205</v>
       </c>
-      <c r="B50" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="C50" s="0" t="s">
+      <c r="B50" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C50" s="2" t="s">
         <v>206</v>
       </c>
-      <c r="E50" s="0" t="s">
+      <c r="E50" s="2" t="s">
         <v>207</v>
       </c>
-      <c r="F50" s="0" t="s">
+      <c r="F50" s="2" t="s">
         <v>208</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="0" t="s">
+      <c r="A51" s="2" t="s">
         <v>209</v>
       </c>
-      <c r="B51" s="0" t="s">
-        <v>45</v>
-      </c>
-      <c r="C51" s="0" t="s">
+      <c r="B51" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="C51" s="2" t="s">
         <v>210</v>
       </c>
-      <c r="E51" s="0" t="s">
+      <c r="E51" s="2" t="s">
         <v>211</v>
       </c>
-      <c r="F51" s="0" t="s">
+      <c r="F51" s="2" t="s">
         <v>212</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="0" t="s">
+      <c r="A52" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="B52" s="0" t="s">
+      <c r="B52" s="2" t="s">
         <v>214</v>
       </c>
-      <c r="C52" s="0" t="s">
+      <c r="C52" s="2" t="s">
         <v>215</v>
       </c>
-      <c r="E52" s="0" t="s">
+      <c r="E52" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="F52" s="0" t="s">
+      <c r="F52" s="2" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="0" t="s">
+      <c r="A53" s="2" t="s">
         <v>216</v>
       </c>
-      <c r="B53" s="0" t="s">
+      <c r="B53" s="2" t="s">
         <v>214</v>
       </c>
-      <c r="C53" s="0" t="s">
+      <c r="C53" s="2" t="s">
         <v>217</v>
       </c>
-      <c r="E53" s="0" t="s">
+      <c r="E53" s="2" t="s">
         <v>218</v>
       </c>
-      <c r="F53" s="0" t="s">
+      <c r="F53" s="2" t="s">
         <v>219</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="0" t="s">
+      <c r="A54" s="2" t="s">
         <v>220</v>
       </c>
-      <c r="B54" s="0" t="s">
+      <c r="B54" s="2" t="s">
         <v>221</v>
       </c>
-      <c r="C54" s="0" t="s">
+      <c r="C54" s="2" t="s">
         <v>222</v>
       </c>
-      <c r="E54" s="0" t="s">
+      <c r="E54" s="2" t="s">
         <v>223</v>
       </c>
-      <c r="F54" s="0" t="s">
+      <c r="F54" s="2" t="s">
         <v>224</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="0" t="s">
+      <c r="A55" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="B55" s="0" t="s">
+      <c r="B55" s="2" t="s">
         <v>221</v>
       </c>
-      <c r="C55" s="0" t="s">
+      <c r="C55" s="2" t="s">
         <v>226</v>
       </c>
-      <c r="E55" s="0" t="s">
+      <c r="E55" s="2" t="s">
         <v>223</v>
       </c>
-      <c r="F55" s="0" t="s">
+      <c r="F55" s="2" t="s">
         <v>224</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="0" t="s">
+      <c r="A56" s="2" t="s">
         <v>227</v>
       </c>
-      <c r="B56" s="0" t="s">
+      <c r="B56" s="2" t="s">
         <v>221</v>
       </c>
-      <c r="C56" s="0" t="s">
+      <c r="C56" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="E56" s="0" t="s">
+      <c r="E56" s="2" t="s">
         <v>229</v>
       </c>
-      <c r="F56" s="0" t="s">
+      <c r="F56" s="2" t="s">
         <v>230</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="0" t="s">
+      <c r="A57" s="2" t="s">
         <v>231</v>
       </c>
-      <c r="B57" s="0" t="s">
+      <c r="B57" s="2" t="s">
         <v>221</v>
       </c>
-      <c r="C57" s="0" t="s">
+      <c r="C57" s="2" t="s">
         <v>232</v>
       </c>
-      <c r="E57" s="0" t="s">
+      <c r="E57" s="2" t="s">
         <v>233</v>
       </c>
-      <c r="F57" s="0" t="s">
+      <c r="F57" s="2" t="s">
         <v>234</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="0" t="s">
+      <c r="A58" s="2" t="s">
         <v>235</v>
       </c>
-      <c r="B58" s="0" t="s">
+      <c r="B58" s="2" t="s">
         <v>221</v>
       </c>
-      <c r="C58" s="0" t="s">
+      <c r="C58" s="2" t="s">
         <v>236</v>
       </c>
-      <c r="E58" s="0" t="s">
+      <c r="E58" s="2" t="s">
         <v>233</v>
       </c>
-      <c r="F58" s="0" t="s">
+      <c r="F58" s="2" t="s">
         <v>234</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="0" t="s">
+      <c r="A59" s="2" t="s">
         <v>237</v>
       </c>
-      <c r="B59" s="0" t="s">
+      <c r="B59" s="2" t="s">
         <v>221</v>
       </c>
-      <c r="C59" s="0" t="s">
+      <c r="C59" s="2" t="s">
         <v>238</v>
       </c>
-      <c r="E59" s="0" t="s">
+      <c r="E59" s="2" t="s">
         <v>239</v>
       </c>
-      <c r="F59" s="0" t="s">
+      <c r="F59" s="2" t="s">
         <v>240</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="0" t="s">
+      <c r="A60" s="2" t="s">
         <v>241</v>
       </c>
-      <c r="B60" s="0" t="s">
+      <c r="B60" s="2" t="s">
         <v>242</v>
       </c>
-      <c r="C60" s="0" t="s">
+      <c r="C60" s="2" t="s">
         <v>243</v>
       </c>
-      <c r="E60" s="0" t="s">
-        <v>244</v>
-      </c>
-      <c r="F60" s="0" t="s">
+      <c r="E60" s="2" t="s">
+        <v>298</v>
+      </c>
+      <c r="F60" s="2" t="s">
         <v>245</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="16.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="0" t="s">
+      <c r="A61" s="2" t="s">
         <v>246</v>
       </c>
-      <c r="B61" s="0" t="s">
+      <c r="B61" s="2" t="s">
         <v>242</v>
       </c>
-      <c r="C61" s="0" t="s">
+      <c r="C61" s="2" t="s">
         <v>247</v>
       </c>
-      <c r="E61" s="0" t="s">
+      <c r="E61" s="2" t="s">
         <v>248</v>
       </c>
-      <c r="F61" s="0" t="s">
+      <c r="F61" s="2" t="s">
         <v>249</v>
       </c>
     </row>

</xml_diff>